<commit_message>
credito nota de venta
</commit_message>
<xml_diff>
--- a/public/formats/color_talla_compras.xlsx
+++ b/public/formats/color_talla_compras.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>COLOR</t>
   </si>
@@ -33,6 +33,9 @@
   </si>
   <si>
     <t>STOCK</t>
+  </si>
+  <si>
+    <t>PRECIO</t>
   </si>
 </sst>
 </file>
@@ -351,10 +354,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -364,50 +367,53 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">

</xml_diff>